<commit_message>
Add scheduler to run main.py at 3:20 PM IST
</commit_message>
<xml_diff>
--- a/Input/search_query.xlsx
+++ b/Input/search_query.xlsx
@@ -5,23 +5,29 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\Media-Monitoring\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\Media-Monitoring\Input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2D3E366-1909-46CE-83F3-F872A168DBAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E3C42D6-F4A1-454D-98F0-78AFAAF51BCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Devendra Fadnavis" sheetId="1" r:id="rId1"/>
-    <sheet name="Eknath Shinde" sheetId="7" r:id="rId2"/>
-    <sheet name="Prakash Abitkar" sheetId="6" r:id="rId3"/>
-    <sheet name="Ravindra Chavan" sheetId="3" r:id="rId4"/>
-    <sheet name="Ashish Shelar" sheetId="4" r:id="rId5"/>
-    <sheet name="Chandrakant Patil" sheetId="8" r:id="rId6"/>
-    <sheet name="Chandrashekhar Bawankule" sheetId="9" r:id="rId7"/>
-    <sheet name="Siddharth Shirole" sheetId="5" r:id="rId8"/>
+    <sheet name="DF Birthday" sheetId="10" r:id="rId1"/>
+    <sheet name="Dhankar Resignation" sheetId="11" r:id="rId2"/>
+    <sheet name="Devendra Fadnavis" sheetId="1" r:id="rId3"/>
+    <sheet name="Eknath Shinde" sheetId="7" r:id="rId4"/>
+    <sheet name="Prakash Abitkar" sheetId="6" r:id="rId5"/>
+    <sheet name="Ravindra Chavan" sheetId="3" r:id="rId6"/>
+    <sheet name="Ashish Shelar" sheetId="4" r:id="rId7"/>
+    <sheet name="Chandrakant Patil" sheetId="8" r:id="rId8"/>
+    <sheet name="Chandrashekhar Bawankule" sheetId="9" r:id="rId9"/>
+    <sheet name="Siddharth Shirole" sheetId="5" r:id="rId10"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'DF Birthday'!$A$1:$A$76</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Dhankar Resignation'!$A$1:$A$76</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -43,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="447" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="599" uniqueCount="566">
   <si>
     <t>devendra fadnavis</t>
   </si>
@@ -1291,13 +1297,463 @@
   </si>
   <si>
     <t>ravindra chavan latest news</t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस वाढदिवस साजरा  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस वाढदिवस सेवादिवस  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस वाढदिवस पुणे उपक्रम  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस वाढदिवस मुख्यमंत्री सहाय्यता निधी  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस वाढदिवस शुभेच्छा  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस वाढदिवस बातम्या महाराष्ट्र  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस वाढदिवस दान कार्यक्रम  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस वाढदिवस गडचिरोली  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस वाढदिवस सामाजिक कार्य  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस वाढदिवस फोटो व्हिडिओ  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस वाढदिवस भाजप कार्यकर्ते  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस वाढदिवस नागपूर  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस वाढदिवस अमृता फडणवीस  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस वाढदिवस रक्तदान शिबिर  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस वाढदिवस समाजसेवा  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस वाढदिवस पायाभूत सुविधा उपक्रम  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस वाढदिवस पर्यावरण संरक्षण  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस वाढदिवस हरित महाराष्ट्र  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस वाढदिवस जलयुक्त शिवार  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस वाढदिवस गडचिरोली वृक्षारोपण  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस वाढदिवस स्मार्ट सिटी प्रकल्प  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस वाढदिवस महामार्ग विकास  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस वाढदिवस शाश्वत विकास  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस वाढदिवस सौर ऊर्जा योजना  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस वाढदिवस समृद्धी महामार्ग  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस जन्मदिन उत्सव  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस जन्मदिन सेवा दिवस  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस जन्मदिन पुणे कार्यक्रम  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस जन्मदिन मुख्यमंत्री राहत कोष  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस जन्मदिन शुभकामनाएं  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस जन्मदिन समाचार महाराष्ट्र  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस जन्मदिन चैरिटी इवेंट  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस जन्मदिन गडचिरोली  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस जन्मदिन सामाजिक कार्य  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस जन्मदिन फोटो वीडियो  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस जन्मदिन भाजपा कार्यकर्ता  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस जन्मदिन नागपुर  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस जन्मदिन अमृता फडणवीस  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस जन्मदिन रक्तदान शिविर  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस जन्मदिन नरेंद्र मोदी शुभकामनाएं  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस जन्मदिन बुनियादी ढांचा पहल  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस जन्मदिन पर्यावरण संरक्षण  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस जन्मदिन हरित महाराष्ट्र  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस जन्मदिन जलयुक्त शिविर  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस जन्मदिन गडचिरोली वृक्षारोपण  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस जन्मदिन स्मार्ट सिटी परियोजना  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस जन्मदिन महामार्ग विकास  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस जन्मदिन सतत विकास  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस जन्मदिन सौर ऊर्जा योजना  </t>
+  </si>
+  <si>
+    <t>देवेंद्र फडणवीस जन्मदिन समृद्धि महामार्ग  </t>
+  </si>
+  <si>
+    <t>Devendra Fadnavis birthday celebration  </t>
+  </si>
+  <si>
+    <t>Devendra Fadnavis birthday Seva Diwas  </t>
+  </si>
+  <si>
+    <t>Devendra Fadnavis birthday Pune events  </t>
+  </si>
+  <si>
+    <t>Devendra Fadnavis birthday Chief Minister Relief Fund  </t>
+  </si>
+  <si>
+    <t>Devendra Fadnavis birthday wishes site:x.com  </t>
+  </si>
+  <si>
+    <t>Devendra Fadnavis birthday Maharashtra news  </t>
+  </si>
+  <si>
+    <t>Devendra Fadnavis birthday charity programs  </t>
+  </si>
+  <si>
+    <t>Devendra Fadnavis birthday Gadchiroli  </t>
+  </si>
+  <si>
+    <t>Devendra Fadnavis birthday social initiatives  </t>
+  </si>
+  <si>
+    <t>Devendra Fadnavis birthday photos videos  </t>
+  </si>
+  <si>
+    <t>Devendra Fadnavis birthday BJP workers  </t>
+  </si>
+  <si>
+    <t>Devendra Fadnavis birthday Nagpur events  </t>
+  </si>
+  <si>
+    <t>Devendra Fadnavis birthday Amruta Fadnavis  </t>
+  </si>
+  <si>
+    <t>Devendra Fadnavis birthday blood donation camp  </t>
+  </si>
+  <si>
+    <t>Devendra Fadnavis birthday Narendra Modi wishes  </t>
+  </si>
+  <si>
+    <t>Devendra Fadnavis birthday infrastructure initiatives  </t>
+  </si>
+  <si>
+    <t>Devendra Fadnavis birthday environmental efforts  </t>
+  </si>
+  <si>
+    <t>Devendra Fadnavis birthday Green Maharashtra  </t>
+  </si>
+  <si>
+    <t>Devendra Fadnavis birthday Jalyukt Shivar  </t>
+  </si>
+  <si>
+    <t>Devendra Fadnavis birthday Gadchiroli tree plantation  </t>
+  </si>
+  <si>
+    <t>Devendra Fadnavis birthday Smart City projects  </t>
+  </si>
+  <si>
+    <t>Devendra Fadnavis birthday highway development  </t>
+  </si>
+  <si>
+    <t>Devendra Fadnavis birthday sustainable development  </t>
+  </si>
+  <si>
+    <t>Devendra Fadnavis birthday solar energy initiatives  </t>
+  </si>
+  <si>
+    <t>Devendra Fadnavis birthday Samruddhi Expressway</t>
+  </si>
+  <si>
+    <t>जगदीप धनखर उपराष्ट्रपती राजीनामा  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर राजीनामा आरोग्य कारण  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर राजीनामा राज्यसभा सभापती  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर राजीनामा बातम्या site:x.com  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर राजीनामा 2025 महाराष्ट्र  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर राजीनामा नरेंद्र मोदी प्रतिक्रिया  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर राजीनामा काँग्रेस टीका  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर राजीनामा पश्चिम बंगाल  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर राजीनामा राजकीय अटकळ  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर राजीनामा राष्ट्रपती द्रौपदी मुर्मू  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर राजीनामा निवडणूक आयोग  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर राजीनामा जयराम रमेश  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर राजीनामा न्यायपालिका वाद  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर राजीनामा नितीश कुमार अटकळ  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर राजीनामा संसद मॉन्सून सत्र  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर राजीनामा बिजेपी रणनीती  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर राजीनामा विरोधी पक्ष प्रतिक्रिया  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर राजीनामा राजस्थान कनेक्शन  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर राजीनामा किसान पुत्र  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर राजीनामा हरिवंश अटकळ  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर राजीनामा संसद व्यवसाय सल्लागार समिती  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर राजीनामा यशवंत वर्मा प्रकरण  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर राजीनामा दिल्ली अँगियोप्लास्टी  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर राजीनामा राजकीय षडयंत्र  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर राजीनामा उपसभापती जबाबदारी  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर उपराष्ट्रपति इस्तीफा  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर इस्तीफा स्वास्थ्य कारण  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर इस्तीफा राज्यसभा अध्यक्ष  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर इस्तीफा समाचार site:x.com  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर इस्तीफा 2025 महाराष्ट्र  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर इस्तीफा नरेंद्र मोदी प्रतिक्रिया  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर इस्तीफा कांग्रेस आलोचना  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर इस्तीफा पश्चिम बंगाल  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर इस्तीफा राजनीतिक अटकलें  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर इस्तीफा राष्ट्रपति द्रौपदी मुर्मू  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर इस्तीफा चुनाव आयोग  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर इस्तीफा जयराम रमेश  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर इस्तीफा न्यायपालिका विवाद  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर इस्तीफा नीतीश कुमार अटकलें  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर इस्तीफा संसद मॉनसून सत्र  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर इस्तीफा बीजेपी रणनीति  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर इस्तीफा विपक्षी प्रतिक्रिया  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर इस्तीफा राजस्थान कनेक्शन  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर इस्तीफा किसान पुत्र  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर इस्तीफा हरिवंश अटकलें  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर इस्तीफा संसद व्यवसाय सलाहकार समिति  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर इस्तीफा यशवंत वर्मा मामला  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर इस्तीफा दिल्ली एंजियोप्लास्टी  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर इस्तीफा राजनीतिक साजिश  </t>
+  </si>
+  <si>
+    <t>जगदीप धनखर इस्तीफा उपाध्यक्ष जिम्मेदारी  </t>
+  </si>
+  <si>
+    <t>Jagdeep Dhankhar Vice President resignation  </t>
+  </si>
+  <si>
+    <t>Jagdeep Dhankhar resignation health reasons  </t>
+  </si>
+  <si>
+    <t>Jagdeep Dhankhar resignation Rajya Sabha Chairman  </t>
+  </si>
+  <si>
+    <t>Jagdeep Dhankhar resignation news site:x.com  </t>
+  </si>
+  <si>
+    <t>Jagdeep Dhankhar resignation 2025 Maharashtra  </t>
+  </si>
+  <si>
+    <t>Jagdeep Dhankhar resignation Narendra Modi reaction  </t>
+  </si>
+  <si>
+    <t>Jagdeep Dhankhar resignation Congress criticism  </t>
+  </si>
+  <si>
+    <t>Jagdeep Dhankhar resignation West Bengal  </t>
+  </si>
+  <si>
+    <t>Jagdeep Dhankhar resignation political speculation  </t>
+  </si>
+  <si>
+    <t>Jagdeep Dhankhar resignation President Droupadi Murmu  </t>
+  </si>
+  <si>
+    <t>Jagdeep Dhankhar resignation Election Commission  </t>
+  </si>
+  <si>
+    <t>Jagdeep Dhankhar resignation Jairam Ramesh  </t>
+  </si>
+  <si>
+    <t>Jagdeep Dhankhar resignation judiciary controversy  </t>
+  </si>
+  <si>
+    <t>Jagdeep Dhankhar resignation Nitish Kumar speculation  </t>
+  </si>
+  <si>
+    <t>Jagdeep Dhankhar resignation Parliament Monsoon Session  </t>
+  </si>
+  <si>
+    <t>Jagdeep Dhankhar resignation BJP strategy  </t>
+  </si>
+  <si>
+    <t>Jagdeep Dhankhar resignation opposition reaction  </t>
+  </si>
+  <si>
+    <t>Jagdeep Dhankhar resignation Rajasthan connection  </t>
+  </si>
+  <si>
+    <t>Jagdeep Dhankhar resignation Kisan Putra  </t>
+  </si>
+  <si>
+    <t>Jagdeep Dhankhar resignation Harivansh speculation  </t>
+  </si>
+  <si>
+    <t>Jagdeep Dhankhar resignation Business Advisory Committee  </t>
+  </si>
+  <si>
+    <t>Jagdeep Dhankhar resignation Yashwant Varma case  </t>
+  </si>
+  <si>
+    <t>Jagdeep Dhankhar resignation Delhi angioplasty  </t>
+  </si>
+  <si>
+    <t>Jagdeep Dhankhar resignation political conspiracy  </t>
+  </si>
+  <si>
+    <t>Jagdeep Dhankhar resignation Deputy Chairman duties</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1309,6 +1765,20 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF222222"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1331,14 +1801,18 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1616,6 +2090,1200 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBAA2A48-F74A-428E-A474-E7E2B0224AE2}">
+  <dimension ref="A1:A76"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A17" s="2" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A18" s="2" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A19" s="2" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A20" s="2" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A21" s="2" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A22" s="2" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A23" s="2" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A24" s="2" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A25" s="2" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A26" s="2" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A27" s="2" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A28" s="2" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A29" s="2" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A30" s="2" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A31" s="2" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A32" s="2" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A33" s="2" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A34" s="2" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A35" s="2" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A36" s="2" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A37" s="2" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A38" s="2" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A39" s="2" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A40" s="2" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A41" s="2" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A42" s="2" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A43" s="2" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A44" s="2" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A45" s="2" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A46" s="2" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A47" s="2" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A48" s="2" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A49" s="2" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A50" s="2" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A51" s="2" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A52" s="2" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A53" s="2" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A54" s="2" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A55" s="2" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A56" s="3" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A57" s="2" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A58" s="2" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A59" s="2" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A60" s="2" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A61" s="2" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A62" s="2" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A63" s="2" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A64" s="2" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A65" s="2" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A66" s="2" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A67" s="2" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A68" s="2" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A69" s="2" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A70" s="2" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A71" s="2" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A72" s="2" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A73" s="2" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A74" s="2" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A75" s="2" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A76" s="2" t="s">
+        <v>490</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A56" r:id="rId1" display="http://x.com/" xr:uid="{D7EEFFD4-6C2C-47EF-BE34-7E2CA27797F0}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86D4577D-FE10-42FD-B10A-D28414797A5F}">
+  <dimension ref="A1:A79"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A64" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A65" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A66" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A67" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A68" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A69" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A70" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A71" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A72" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A73" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A74" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A75" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A76" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A77" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A78" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A79" t="s">
+        <v>243</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB4A1374-30FD-4B53-B704-0480A0FBF33D}">
+  <dimension ref="A1:A76"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A17" s="2" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A18" s="2" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A19" s="2" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A20" s="2" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A21" s="2" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A22" s="2" t="s">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A23" s="2" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A24" s="2" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A25" s="2" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A26" s="2" t="s">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A27" s="2" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A28" s="2" t="s">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A29" s="2" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A30" s="3" t="s">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A31" s="2" t="s">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A32" s="2" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A33" s="2" t="s">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A34" s="2" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A35" s="2" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A36" s="2" t="s">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A37" s="2" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A38" s="2" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A39" s="2" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A40" s="2" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A41" s="2" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A42" s="2" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A43" s="2" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A44" s="2" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A45" s="2" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A46" s="2" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A47" s="2" t="s">
+        <v>536</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A48" s="2" t="s">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A49" s="2" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A50" s="2" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A51" s="2" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A52" s="2" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A53" s="2" t="s">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A54" s="2" t="s">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A55" s="3" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A56" s="2" t="s">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A57" s="2" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A58" s="2" t="s">
+        <v>547</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A59" s="2" t="s">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A60" s="2" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A61" s="2" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A62" s="2" t="s">
+        <v>551</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A63" s="2" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A64" s="2" t="s">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A65" s="2" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A66" s="2" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A67" s="2" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A68" s="2" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A69" s="2" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A70" s="2" t="s">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A71" s="2" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A72" s="2" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A73" s="2" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A74" s="2" t="s">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A75" s="2" t="s">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A76" s="2" t="s">
+        <v>565</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A5" r:id="rId1" display="http://x.com/" xr:uid="{E8684EE2-6127-4F55-B488-0B95874D9B35}"/>
+    <hyperlink ref="A30" r:id="rId2" display="http://x.com/" xr:uid="{6638835F-4F41-4FA3-AEEA-1357500FCB21}"/>
+    <hyperlink ref="A55" r:id="rId3" display="http://x.com/" xr:uid="{BC0BA897-4E54-4D91-8260-6ED872577DBA}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:A105"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2153,7 +3821,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E8F7DD1D-0DFC-440F-988C-050CA65FFA2F}">
   <dimension ref="A1:A185"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3088,7 +4756,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C494B66-AEA5-4CCE-888E-96E7151CA2B5}">
   <dimension ref="A1:A48"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3338,7 +5006,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13BB4D98-1E3A-4E3C-ACBA-9B32A23C1612}">
   <dimension ref="A1:A14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3421,7 +5089,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20836306-9997-450D-A55C-BA5D93912EB9}">
   <dimension ref="A1:A14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3504,7 +5172,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3999BA3D-14F7-4974-A4C1-C319E42C52A3}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3519,7 +5187,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C323B3F7-4FF2-40F4-B949-CB50AFBFD4BF}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3532,409 +5200,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86D4577D-FE10-42FD-B10A-D28414797A5F}">
-  <dimension ref="A1:A79"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A30" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A32" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A34" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A35" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A36" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A37" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A38" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A39" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A40" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A41" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A42" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A43" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A44" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A45" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A46" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A47" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A48" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A49" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A50" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A51" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A52" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A53" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A54" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A55" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A56" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A57" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A58" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A59" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A60" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A61" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A62" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A63" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A64" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A65" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A66" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A67" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A68" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A69" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A70" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A71" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A72" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A73" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A74" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A75" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A76" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A77" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A78" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A79" t="s">
-        <v>243</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>